<commit_message>
Changed Rock Type Mapping in 1.1_Wrapper for REFLECT, MDPI Tibet, CAES2014 and ALPS. More following - used Rock-Type_Manuel Excel
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/thermal_springs_alps_with_HF_estimates.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/thermal_springs_alps_with_HF_estimates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69B98BA-085F-4DF1-9DCB-B8927DBB9308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SHEET1" sheetId="1" r:id="rId1"/>

</xml_diff>